<commit_message>
fix: pay item rewards larger than one stack #723
- character: make a DSL item reward in pieces of the item capacity
- items: refuse a bundle reward or exchange that does not fit in one stack
- reward table: add the test.reward.split and test.reward.over rewards
- integration tests: add the reward split scenario to the item test
</commit_message>
<xml_diff>
--- a/resources/table/reward.xlsx
+++ b/resources/table/reward.xlsx
@@ -1,111 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381FD236-75BF-40C0-8608-2739D5090614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="reward" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reward" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
-  <si>
-    <t>id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>*string</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>server</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dsl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[dsl]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>quest1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>quest1.step.1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>quest1.step.3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>item(3014, 201)
-money(10000)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>item(3014, 150)
-money(10000)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>item(3014, 100)
-exp(10000)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -121,34 +59,94 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -448,65 +446,119 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8D9647-70DB-4352-ABD3-4D2F60838B15}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="11.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.75" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="1"/>
+    <col width="11.375" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="17.75" customWidth="1" style="1" min="2" max="2"/>
+    <col width="9" customWidth="1" style="1" min="3" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>*string</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>[dsl]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="27" customHeight="1" s="3">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>quest1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>item(3014, 201)
+money(10000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27" customHeight="1" s="3">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>quest1.step.1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>item(3014, 100)
+exp(10000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27" customHeight="1" s="3">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>quest1.step.3</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>item(3014, 150)
+money(10000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>test.reward.split</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>item(75, 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>test.reward.over</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>item(3014, 250)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>